<commit_message>
feat: add new game data and player statistics for games 3 and 4; update localization and styles
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/data/工作簿1.xlsx
+++ b/data/工作簿1.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lizuan/program/basketball/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C51DCFF-9E95-C34F-AB01-7C21270C46BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832393F2-432E-4B4C-AE1B-0B01F223796C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="620" windowWidth="28100" windowHeight="16280" activeTab="1" xr2:uid="{D6A172F3-6A8A-304E-83AA-40110FEEC815}"/>
+    <workbookView xWindow="340" yWindow="620" windowWidth="28100" windowHeight="16280" activeTab="2" xr2:uid="{D6A172F3-6A8A-304E-83AA-40110FEEC815}"/>
   </bookViews>
   <sheets>
     <sheet name="Game1" sheetId="1" r:id="rId1"/>
     <sheet name="Game2" sheetId="2" r:id="rId2"/>
+    <sheet name="Game3" sheetId="3" r:id="rId3"/>
+    <sheet name="Game4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="107">
   <si>
     <t>Player</t>
   </si>
@@ -256,6 +258,111 @@
   </si>
   <si>
     <t>14</t>
+  </si>
+  <si>
+    <t>1(1)</t>
+  </si>
+  <si>
+    <t>13(7)</t>
+  </si>
+  <si>
+    <t>3(1)</t>
+  </si>
+  <si>
+    <t>Chai</t>
+  </si>
+  <si>
+    <t>7(5)</t>
+  </si>
+  <si>
+    <t>14/40</t>
+  </si>
+  <si>
+    <t>20/57</t>
+  </si>
+  <si>
+    <t>33(16)</t>
+  </si>
+  <si>
+    <t>2/10</t>
+  </si>
+  <si>
+    <t>3/14</t>
+  </si>
+  <si>
+    <t>4/10</t>
+  </si>
+  <si>
+    <t>4/13</t>
+  </si>
+  <si>
+    <t>9/15</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>1/1</t>
+  </si>
+  <si>
+    <t>1/2</t>
+  </si>
+  <si>
+    <t>6/17</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>0/5</t>
+  </si>
+  <si>
+    <t>6(1)</t>
+  </si>
+  <si>
+    <t>0/6</t>
+  </si>
+  <si>
+    <t>10(3)</t>
+  </si>
+  <si>
+    <t>8(3)</t>
+  </si>
+  <si>
+    <t>12/34</t>
+  </si>
+  <si>
+    <t>13/46</t>
+  </si>
+  <si>
+    <t>32(7)</t>
+  </si>
+  <si>
+    <t>2/6</t>
+  </si>
+  <si>
+    <t>2/11</t>
+  </si>
+  <si>
+    <t>1/10</t>
+  </si>
+  <si>
+    <t>6/13</t>
+  </si>
+  <si>
+    <t>3/5</t>
+  </si>
+  <si>
+    <t>1/12</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>8</t>
   </si>
 </sst>
 </file>
@@ -1206,4 +1313,608 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D28E7E44-BE07-D84F-843B-2901EDE13A7F}">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69D6BEBF-CBCE-1447-A6E5-F8C269118345}">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>